<commit_message>
feat(TASK-043): add economic_layer sheet to demo dataset (derived realistic values)
</commit_message>
<xml_diff>
--- a/data/sample/sample_planning.xlsx
+++ b/data/sample/sample_planning.xlsx
@@ -11,6 +11,7 @@
     <sheet name="product_matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="labs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="phase_capacity" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="economic_layer" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1376,4 +1377,200 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>assigned_lab</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>product_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>standard_hourly_cost_eur</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>overtime_multiplier</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>overhead_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>setup_cost_eur</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ORD-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Giacca</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ORD-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pantalone</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ORD-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Giacca</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ORD-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pantalone</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ORD-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Giacca</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>